<commit_message>
Fix translation fallback and export safety
</commit_message>
<xml_diff>
--- a/DataTables/translations_managed.xlsx
+++ b/DataTables/translations_managed.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="UI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Herbs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Formulas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Diseases" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="NPC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herbs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -227,7 +227,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="NPCTranslations" displayName="NPCTranslations" ref="A1:C301" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="NPCTranslations" displayName="NPCTranslations" ref="A1:C302" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" name="keys"/>
     <tableColumn id="2" name="zh_CN"/>
@@ -24497,7 +24497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C301"/>
+  <dimension ref="A1:C302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -29622,6 +29622,23 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" s="7" t="inlineStr">
+        <is>
+          <t>UI_NPC_GENERIC_SYMPTOM</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>身体不适</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>feeling unwell</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>